<commit_message>
Add 17 more competitors to spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6bcYix3HsyTfpCARdd46p
</commit_message>
<xml_diff>
--- a/summary-ai-competitors.xlsx
+++ b/summary-ai-competitors.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1191,9 +1191,979 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Smart Noter - AI Note Taker</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Deep Flow Apps</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>5M+</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (AppBrain similar-apps list); package ID not found</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>MeetGeek: AI Note Taker</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>MeetGeek</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>100K+</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (AppBrain)</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/dev/MeetGeek%3A+AI+Note+Taker.+Transcribe+Speech+to+Text/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Transcribe Audio To Text</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DKTLabs</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>500K+</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (AppBrain similar-apps list)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AI Transcript: Audio to Text</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Appzys</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>10K+</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (AppBrain similar-apps list)</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>NoteQA - AI Audio Transcription</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Pixster Studio</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>10K+</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2.2★</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.pixsterstudio.transcribe</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (AppBrain); package ID from AppBrain URL</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/app/noteqa-ai-audio-transcription/com.pixsterstudio.transcribe</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Audionotes</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Audionotes</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>$70/yr Personal; $130/yr Pro</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>4.8★ (per blog)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Android-focused</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Blog claim, unverified</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.audionotes.app/blog/best-note-taking-apps-for-android</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Fireflies</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Fireflies.ai</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Mobile + web (unverified)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Named in roundups only</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Krisp</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Krisp</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Free trial, paid tiers</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Named in roundups only</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ScreenApp</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ScreenApp</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Mobile capture + web</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Named in roundups only</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://screenapp.io/nl/blog/best-mobile-ai-note-taking-apps</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Granola</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Granola</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Mac, iOS (not Android per roundup)</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Named in roundups only</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Fathom</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Fathom</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Free tier</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://toolradar.com/alternatives/buddy-ai-note</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Read.ai</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Read.ai</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://toolradar.com/alternatives/buddy-ai-note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Sembly AI</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Sembly</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://toolradar.com/alternatives/buddy-ai-note</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Supernormal</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Supernormal</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://toolradar.com/alternatives/buddy-ai-note</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Coconote</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Coconote</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://toolradar.com/alternatives/coconote</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Mem</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Mem</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Named in directory lists only</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.toolfinder.com/best/mem-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>VoicePen: AI Note Taker</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VoicePen</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>AppBrain iOS page; no Android found</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/appstore/ai-note-taker-voicepen/ios-6462815872</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1205,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1239,6 +2209,13 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Round 2 rows come from roundup blogs and AppBrain pages; roundup-only apps have no verified data. Rows 14+ are unranked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Labhouse revenue, deal findings and valuation model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6bcYix3HsyTfpCARdd46p
</commit_message>
<xml_diff>
--- a/summary-ai-competitors.xlsx
+++ b/summary-ai-competitors.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitors" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labhouse findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +36,12 @@
     <font>
       <color rgb="000563C1"/>
       <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000000FF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -60,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -71,6 +80,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +550,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1M–10M (AppBrain, all Labhouse apps); one tracker ~2.3M (unverified)</t>
+          <t>1M+ (Google Play bucket per search); AppBrain ~1.5M est.; one tracker ~2.3M (unverified)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -560,7 +575,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Package ID confirmed via Chrome-Stats: https://chrome-stats.com/d/io.labhouse.audioapp ; Play page itself not opened</t>
+          <t>Package ID confirmed via Chrome-Stats: https://chrome-stats.com/d/io.labhouse.audioapp ; Play page itself not opened | Play: https://play.google.com/store/apps/details?id=io.labhouse.audioapp ; AppBrain: https://www.appbrain.com/app/summary-ai-note-taker/io.labhouse.audioapp</t>
         </is>
       </c>
     </row>
@@ -2175,6 +2190,585 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Source / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Summary AI total, per month</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>~$700K</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Estimated (unverified, likely gross)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ScreensDesign (prior research)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Summary AI Android, per month</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>~$30K</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://trendapps.dev/app/android/io-labhouse-audioapp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Labhouse 2024 sales</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Not public</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Hidden</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Accounts filed; figures paywalled (Infonif/eInforma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Downloads</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Android bucket (Google Play)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>1M+</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (search result, page not opened)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.labhouse.audioapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Downloads</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Android total / last 30 days (AppBrain)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>~1.5M / ~390K</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.appbrain.com/app/summary-ai-note-taker/io.labhouse.audioapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Downloads</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Android last 30 days (TrendApps)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>~100K</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Estimated (conflicts with AppBrain)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://trendapps.dev/app/android/io-labhouse-audioapp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Ratings</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>iOS ratings count</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>~54K (earlier note: 31.9K)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Conflicting</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/us/app/summary-ai-note-taker/id6670175056</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Deals</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Acquisition offer / news</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Searched news and profiles; no report</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Deals</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Outside funding</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Registry shows a capital increase, investor not named: https://infonif.economia3.com/ficha-empresa/labhouse-mobile-sl</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Deals</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Martos personal investing</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2 investments (Baobab Ventures)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://pitchbook.com/profiles/investor/232475-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Spain sales rank 2024</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>50,352nd; 2025 result negative</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Sourced (amount not shown)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://ranking-empresas.eleconomista.es/LABHOUSE-MOBILE.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Apps</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Summary AI, Invoice Fly, Cleaner GO, Super Chat, Notespace</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Search results; 100M+ downloads is a company claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>VALUATION MODEL (estimate; inputs in blue can be edited)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gross revenue / yr ($)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>8400000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Store fee low</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Store fee high</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rev multiple low</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rev multiple high</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EBITDA margin low</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EBITDA margin high</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EBITDA multiple low</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EBITDA multiple high</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Net revenue low</t>
+        </is>
+      </c>
+      <c r="C26" s="9">
+        <f>C16*(1-C18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Net revenue high</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>C16*(1-C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Revenue-multiple value low</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>C26*C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Revenue-multiple value high</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>C27*C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EBITDA low</t>
+        </is>
+      </c>
+      <c r="C30" s="9">
+        <f>C26*C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EBITDA high</t>
+        </is>
+      </c>
+      <c r="C31" s="9">
+        <f>C27*C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EBITDA-multiple value low</t>
+        </is>
+      </c>
+      <c r="C32" s="9">
+        <f>C30*C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EBITDA-multiple value high</t>
+        </is>
+      </c>
+      <c r="C33" s="9">
+        <f>C31*C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Overlap range (estimate)</t>
+        </is>
+      </c>
+      <c r="C34" s="9">
+        <f>MAX(C28,C32)</f>
+        <v/>
+      </c>
+      <c r="D34" s="9">
+        <f>MIN(C29,C33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Not a valuation opinion: based on an unverified revenue estimate; no churn or ad-cost data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add offline competitors, Android data and ANotes similarity scores
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6bcYix3HsyTfpCARdd46p
</commit_message>
<xml_diff>
--- a/summary-ai-competitors.xlsx
+++ b/summary-ai-competitors.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -86,6 +86,9 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -465,6 +468,8 @@
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,6 +528,16 @@
           <t>Source / notes</t>
         </is>
       </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>ANotes similarity /10 (my judgment)</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -578,6 +593,14 @@
           <t>Package ID confirmed via Chrome-Stats: https://chrome-stats.com/d/io.labhouse.audioapp ; Play page itself not opened | Play: https://play.google.com/store/apps/details?id=io.labhouse.audioapp ; AppBrain: https://www.appbrain.com/app/summary-ai-note-taker/io.labhouse.audioapp</t>
         </is>
       </c>
+      <c r="L2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Voice to transcript to summary on Android; cloud, subscription</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -635,6 +658,14 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Cloud meeting transcription</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -692,6 +723,12 @@
           <t>https://screensdesign.com/apps/plaud-ai-voice-recorder/</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -749,6 +786,14 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Cloud meeting transcription</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -806,6 +851,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -835,32 +886,40 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>100K+</t>
+          <t>100K+ (AppBrain/Play bucket); ~190K lifetime est.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~3.87★ / ~2.5K (AppBrain)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Android (iOS unconfirmed)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>Android, iOS (cloud-based per competitor blog)</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.app.voicenotes</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Prior research; Play link not verified</t>
+          <t>Tracker data (AppBrain, Chrome-Stats); package ID from trackers, Play page not opened</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Prior research (user-supplied)</t>
+          <t>https://www.appbrain.com/app/voicenotes/com.app.voicenotes ; developer Coping Hard Inc.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Voice-first notes, Android; cloud, subscription</t>
         </is>
       </c>
     </row>
@@ -920,6 +979,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -977,6 +1042,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1034,6 +1105,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1091,6 +1168,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1148,6 +1231,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1205,6 +1294,12 @@
           <t>Prior research (user-supplied)</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1262,6 +1357,12 @@
           <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1319,6 +1420,12 @@
           <t>https://www.appbrain.com/dev/MeetGeek%3A+AI+Note+Taker.+Transcribe+Speech+to+Text/</t>
         </is>
       </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1376,6 +1483,12 @@
           <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
         </is>
       </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1433,6 +1546,12 @@
           <t>https://www.appbrain.com/app/voice-recorder-ai-transcribe/kr.co.neoandroid.recoder</t>
         </is>
       </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1490,6 +1609,12 @@
           <t>https://www.appbrain.com/app/noteqa-ai-audio-transcription/com.pixsterstudio.transcribe</t>
         </is>
       </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1524,27 +1649,35 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>4.8★ (per blog)</t>
+          <t>~4.77★ / 88 ratings (AppBrain)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Android-focused</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>Android, iOS (cloud AI per vendor)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.labs.audionotes</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Blog claim, unverified</t>
+          <t>Package per SimilarWeb, UNCONFIRMED (AppBrain lists a different developer); installs not found</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>https://www.audionotes.app/blog/best-note-taking-apps-for-android</t>
+          <t>https://www.similarweb.com/ko/app/google/com.labs.audionotes/</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Voice notes, cloud AI, subscription</t>
         </is>
       </c>
     </row>
@@ -1604,6 +1737,14 @@
           <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
         </is>
       </c>
+      <c r="L20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Cloud-first meetings</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1661,6 +1802,12 @@
           <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1718,6 +1865,12 @@
           <t>https://screenapp.io/nl/blog/best-mobile-ai-note-taking-apps</t>
         </is>
       </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1775,6 +1928,14 @@
           <t>https://www.happyscribe.com/blog/best-ai-meeting-note-takers-for-android</t>
         </is>
       </c>
+      <c r="L23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Mac/iOS meetings</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1832,6 +1993,12 @@
           <t>https://toolradar.com/alternatives/buddy-ai-note</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1889,6 +2056,12 @@
           <t>https://toolradar.com/alternatives/buddy-ai-note</t>
         </is>
       </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1946,6 +2119,12 @@
           <t>https://toolradar.com/alternatives/buddy-ai-note</t>
         </is>
       </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2003,6 +2182,12 @@
           <t>https://toolradar.com/alternatives/buddy-ai-note</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2060,6 +2245,12 @@
           <t>https://toolradar.com/alternatives/coconote</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2117,6 +2308,14 @@
           <t>https://www.toolfinder.com/best/mem-alternatives</t>
         </is>
       </c>
+      <c r="L29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>AI notes, not voice-first, no offline</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2172,13 +2371,478 @@
       <c r="K30" s="2" t="inlineStr">
         <is>
           <t>https://www.appbrain.com/appstore/ai-note-taker-voicepen/ios-6462815872</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>not scored (no info)</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Yaps</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Yaps</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Free; Pro $12/mo (vendor)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Android keyboard (+ other platforms)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Vendor claims, unverified: on-device dictation, offline cleanup option</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yaps.ai/android</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Android, on-device dictation + read-aloud; keyboard not notes app</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Whisper: Voice to Text</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>(lazycattle)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Free tier with daily limit; one-time Pro</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.lazycattle.transcribe</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Vendor claims offline, unverified</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.lazycattle.transcribe&amp;hl=en_GB</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Android, claims fully offline; free tier + one-time Pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Whisper Android Speech To Text</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>(signalmaster)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Mixed reviews (UX)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.signalmaster.asr</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Listing says offline Whisper; unverified</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.signalmaster.asr</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Offline Whisper but weak notes UX per reviews</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>VoicePad</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>VoicePad</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>One-time price (vendor)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Android + desktop + iOS</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Vendor claims local Whisper; Play listing not confirmed</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>https://voicepad.tech/offline-speech-to-text/</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Local Whisper, one-time price; Android availability unconfirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Notely Voice</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Open source</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Free (open source)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Android, iOS</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Repo claims on-device Whisper; Play listing not confirmed</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/tosinonikute/NotelyVoice</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Open source, on-device Whisper, Android; closest in approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Hands Free Notes</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Indie dev</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Developer post only; unverified</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://dev.to/turnkit-dev/whisper-on-mobile-is-better-than-i-expected-so-i-built-an-offline-notes-app-41d7</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>On-device voice notes on Android; indie, unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>VoiceScriber AI: Offline Notes</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>VoiceScriber</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>$39.99 one-time; $4.99/mo; $29.99/yr</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>iOS only</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Vendor claims on-device, offline; iOS only</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://apps.apple.com/us/app/voicescriber-ai-offline-notes/id6736822144</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Offline, on-device notes but iOS only</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2769,7 +3433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2810,6 +3474,13 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Round 3: similarity scores are my judgment vs ANotes (offline, on-device, Android, Markdown). Most offline claims are vendor marketing, unverified. Play pages could not be opened from this environment.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add permissions and network notes for offline apps
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6bcYix3HsyTfpCARdd46p
</commit_message>
<xml_diff>
--- a/summary-ai-competitors.xlsx
+++ b/summary-ai-competitors.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -470,6 +470,7 @@
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,6 +539,11 @@
           <t>Why</t>
         </is>
       </c>
+      <c r="N1" s="10" t="inlineStr">
+        <is>
+          <t>Permissions / network notes (unverified)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2444,6 +2450,11 @@
           <t>Android, on-device dictation + read-aloud; keyboard not notes app</t>
         </is>
       </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Vendor says microphone is the only permission, no Accessibility Service; audio stays on device. A Japanese page mentions an Accessibility Service check-in (contradiction, unresolved). INTERNET not addressed; cloud cleanup mode exists. https://www.yaps.ai/blog/yaps-android-app-launch</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2473,7 +2484,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~16 downloads (Chrome-Stats, 2026-08-01; tracker)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2502,11 +2513,16 @@
         </is>
       </c>
       <c r="L32" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Android, claims fully offline; free tier + one-time Pro</t>
+          <t>Claims offline, but tiny reach and no permissions info</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Vendor claims offline, no data collection. No permissions list or privacy policy found. Only ~16 downloads (Chrome-Stats, 2026-08-01). https://chrome-stats.com/d/com.lazycattle.transcribe</t>
         </is>
       </c>
     </row>
@@ -2574,6 +2590,11 @@
           <t>Offline Whisper but weak notes UX per reviews</t>
         </is>
       </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Nothing found for com.signalmaster.asr; treat listing as unverified.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2681,14 +2702,14 @@
           <t>Android, iOS</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>https://f-droid.org/packages/com.module.notelycompose.android/</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Repo claims on-device Whisper; Play listing not confirmed</t>
+          <t>F-Droid listing found (not Play); on-device claim from repo, unverified</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2702,6 +2723,11 @@
       <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Open source, on-device Whisper, Android; closest in approach</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>F-Droid (com.module.notelycompose.android) lists: full network access, microphone foreground service, download-without-notification. Network likely for model download (inference). RECORD_AUDIO/INTERNET not confirmed by name. Source is public, not audited. https://f-droid.org/packages/com.module.notelycompose.android/</t>
         </is>
       </c>
     </row>
@@ -2843,6 +2869,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3433,7 +3460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3481,6 +3508,13 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Permissions notes (round 4): Play Data safety pages and APK manifests could not be opened; all entries are from vendor posts, F-Droid or trackers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>